<commit_message>
Explored other trends in data
</commit_message>
<xml_diff>
--- a/Copper/6. Sensitivity analyses/Plots of HA SA/HA_Sensitivity_Summary.xlsx
+++ b/Copper/6. Sensitivity analyses/Plots of HA SA/HA_Sensitivity_Summary.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t xml:space="preserve">Typology</t>
   </si>
@@ -58,12 +58,6 @@
   </si>
   <si>
     <t xml:space="preserve">50-60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60-70</t>
-  </si>
-  <si>
-    <t xml:space="preserve">70-80</t>
   </si>
   <si>
     <t xml:space="preserve">NP Tribs</t>
@@ -577,86 +571,86 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.00000000160569786788999</v>
+        <v>-0.00000000431212662469429</v>
       </c>
       <c r="D7" t="n">
-        <v>0.000000000262435774373832</v>
+        <v>0.000000000732510674399534</v>
       </c>
       <c r="E7" t="n">
-        <v>-10.8467582014117</v>
+        <v>-39.2443546078952</v>
       </c>
       <c r="F7" t="n">
-        <v>0.14914553379026</v>
+        <v>0.908466087854785</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0499377048516895</v>
+        <v>-0.217024126734495</v>
       </c>
       <c r="H7" t="n">
-        <v>0.000714250344220309</v>
+        <v>0.00633693598334707</v>
       </c>
       <c r="I7" t="n">
-        <v>127</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.00000000126886278102653</v>
+        <v>-0.00000000184125693789807</v>
       </c>
       <c r="D8" t="n">
-        <v>0.000000000201834358210185</v>
+        <v>0.000000000298774498861813</v>
       </c>
       <c r="E8" t="n">
-        <v>-9.7720238460795</v>
+        <v>-28.1862503999904</v>
       </c>
       <c r="F8" t="n">
-        <v>0.125682346459932</v>
+        <v>0.481881337044835</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.0447108124144785</v>
+        <v>-0.143917388131278</v>
       </c>
       <c r="H8" t="n">
-        <v>0.000595900941300992</v>
+        <v>0.00287786577037895</v>
       </c>
       <c r="I8" t="n">
-        <v>127</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.00000000431212662469429</v>
+        <v>-0.00000000102224736035393</v>
       </c>
       <c r="D9" t="n">
-        <v>0.000000000732510674399534</v>
+        <v>0.000000000162168698509139</v>
       </c>
       <c r="E9" t="n">
-        <v>-39.2443546078952</v>
+        <v>-21.9860667878466</v>
       </c>
       <c r="F9" t="n">
-        <v>0.908466087854785</v>
+        <v>0.29777385282192</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.217024126734495</v>
+        <v>-0.107868538314292</v>
       </c>
       <c r="H9" t="n">
-        <v>0.00633693598334707</v>
+        <v>0.00164514860302336</v>
       </c>
       <c r="I9" t="n">
         <v>14</v>
@@ -664,28 +658,28 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.00000000184125693789807</v>
+        <v>-0.000000000650526269084162</v>
       </c>
       <c r="D10" t="n">
-        <v>0.000000000298774498861813</v>
+        <v>0.000000000101814451582528</v>
       </c>
       <c r="E10" t="n">
-        <v>-28.1862503999904</v>
+        <v>-18.0216151340535</v>
       </c>
       <c r="F10" t="n">
-        <v>0.481881337044835</v>
+        <v>0.202070243403988</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.143917388131278</v>
+        <v>-0.0863176783693471</v>
       </c>
       <c r="H10" t="n">
-        <v>0.00287786577037895</v>
+        <v>0.00106509249819166</v>
       </c>
       <c r="I10" t="n">
         <v>14</v>
@@ -693,28 +687,28 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.00000000102224736035393</v>
+        <v>-0.000000000450472994053227</v>
       </c>
       <c r="D11" t="n">
-        <v>0.000000000162168698509139</v>
+        <v>0.0000000000698706871238354</v>
       </c>
       <c r="E11" t="n">
-        <v>-21.9860667878466</v>
+        <v>-15.2693905045291</v>
       </c>
       <c r="F11" t="n">
-        <v>0.29777385282192</v>
+        <v>0.146161932400706</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.107868538314292</v>
+        <v>-0.0719680291788789</v>
       </c>
       <c r="H11" t="n">
-        <v>0.00164514860302336</v>
+        <v>0.000746457703950461</v>
       </c>
       <c r="I11" t="n">
         <v>14</v>
@@ -722,144 +716,144 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.000000000650526269084162</v>
+        <v>-0.0000000101365266565971</v>
       </c>
       <c r="D12" t="n">
-        <v>0.000000000101814451582528</v>
+        <v>0.00000000261414290126978</v>
       </c>
       <c r="E12" t="n">
-        <v>-18.0216151340535</v>
+        <v>-31.4127567413295</v>
       </c>
       <c r="F12" t="n">
-        <v>0.202070243403988</v>
+        <v>0.478777520088047</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.0863176783693471</v>
+        <v>-0.164772519519664</v>
       </c>
       <c r="H12" t="n">
-        <v>0.00106509249819166</v>
+        <v>0.00300877299503251</v>
       </c>
       <c r="I12" t="n">
-        <v>14</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.000000000450472994053227</v>
+        <v>-0.00000000529431734128614</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0000000000698706871238354</v>
+        <v>0.00000000148290068883031</v>
       </c>
       <c r="E13" t="n">
-        <v>-15.2693905045291</v>
+        <v>-23.9286150564038</v>
       </c>
       <c r="F13" t="n">
-        <v>0.146161932400706</v>
+        <v>0.285691448463723</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.0719680291788789</v>
+        <v>-0.119073063016372</v>
       </c>
       <c r="H13" t="n">
-        <v>0.000746457703950461</v>
+        <v>0.00161998195318168</v>
       </c>
       <c r="I13" t="n">
-        <v>14</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.000000000330436535989546</v>
+        <v>-0.0000000032151860050683</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0000000000509237360986556</v>
+        <v>0.000000000929497879865746</v>
       </c>
       <c r="E14" t="n">
-        <v>-13.2467156528484</v>
+        <v>-19.3165293475852</v>
       </c>
       <c r="F14" t="n">
-        <v>0.110673508789087</v>
+        <v>0.190710549440983</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.0617186521199884</v>
+        <v>-0.093332301387409</v>
       </c>
       <c r="H14" t="n">
-        <v>0.000552538727642766</v>
+        <v>0.00102126338610707</v>
       </c>
       <c r="I14" t="n">
-        <v>14</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.000000000252779735760042</v>
+        <v>-0.00000000214170459450046</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0000000000387687930723166</v>
+        <v>0.000000000624174037887801</v>
       </c>
       <c r="E15" t="n">
-        <v>-11.6987825088521</v>
+        <v>-16.1925691927188</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0869515790411032</v>
+        <v>0.136803551247869</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.0540360379390628</v>
+        <v>-0.0767733162364369</v>
       </c>
       <c r="H15" t="n">
-        <v>0.000426754373127797</v>
+        <v>0.000706261241767529</v>
       </c>
       <c r="I15" t="n">
-        <v>14</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.0000000101365266565971</v>
+        <v>-0.00000000152126988823109</v>
       </c>
       <c r="D16" t="n">
-        <v>0.00000000261414290126978</v>
+        <v>0.000000000442614365083958</v>
       </c>
       <c r="E16" t="n">
-        <v>-31.4127567413295</v>
+        <v>-13.9373464420318</v>
       </c>
       <c r="F16" t="n">
-        <v>0.478777520088047</v>
+        <v>0.103091800728416</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.164772519519664</v>
+        <v>-0.0652153796755085</v>
       </c>
       <c r="H16" t="n">
-        <v>0.00300877299503251</v>
+        <v>0.000518793080148642</v>
       </c>
       <c r="I16" t="n">
         <v>98</v>
@@ -867,378 +861,146 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.00000000529431734128614</v>
+        <v>-0.00000000520693650759922</v>
       </c>
       <c r="D17" t="n">
-        <v>0.00000000148290068883031</v>
+        <v>0.00000000041839707087581</v>
       </c>
       <c r="E17" t="n">
-        <v>-23.9286150564038</v>
+        <v>-28.1665669334067</v>
       </c>
       <c r="F17" t="n">
-        <v>0.285691448463723</v>
+        <v>0.381536838631078</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.119073063016372</v>
+        <v>-0.144372698646437</v>
       </c>
       <c r="H17" t="n">
-        <v>0.00161998195318168</v>
+        <v>0.00228015145786663</v>
       </c>
       <c r="I17" t="n">
-        <v>98</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.0000000032151860050683</v>
+        <v>-0.00000000287110789505956</v>
       </c>
       <c r="D18" t="n">
-        <v>0.000000000929497879865746</v>
+        <v>0.000000000232068845738583</v>
       </c>
       <c r="E18" t="n">
-        <v>-19.3165293475852</v>
+        <v>-21.975638509489</v>
       </c>
       <c r="F18" t="n">
-        <v>0.190710549440983</v>
+        <v>0.238732918197057</v>
       </c>
       <c r="G18" t="n">
-        <v>-0.093332301387409</v>
+        <v>-0.108001931629995</v>
       </c>
       <c r="H18" t="n">
-        <v>0.00102126338610707</v>
+        <v>0.00131351800505018</v>
       </c>
       <c r="I18" t="n">
-        <v>98</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.00000000214170459450046</v>
+        <v>-0.00000000182021027054008</v>
       </c>
       <c r="D19" t="n">
-        <v>0.000000000624174037887801</v>
+        <v>0.000000000146852331251988</v>
       </c>
       <c r="E19" t="n">
-        <v>-16.1925691927188</v>
+        <v>-18.0120336902386</v>
       </c>
       <c r="F19" t="n">
-        <v>0.136803551247869</v>
+        <v>0.163853621564138</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.0767733162364369</v>
+        <v>-0.0863491897459432</v>
       </c>
       <c r="H19" t="n">
-        <v>0.000706261241767529</v>
+        <v>0.000859564182326996</v>
       </c>
       <c r="I19" t="n">
-        <v>98</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.00000000152126988823109</v>
+        <v>-0.00000000125729130997135</v>
       </c>
       <c r="D20" t="n">
-        <v>0.000000000442614365083958</v>
+        <v>0.000000000100967193306608</v>
       </c>
       <c r="E20" t="n">
-        <v>-13.9373464420318</v>
+        <v>-15.2593635143343</v>
       </c>
       <c r="F20" t="n">
-        <v>0.103091800728416</v>
+        <v>0.119616550477939</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.0652153796755085</v>
+        <v>-0.071957936590277</v>
       </c>
       <c r="H20" t="n">
-        <v>0.000518793080148642</v>
+        <v>0.00060818545475409</v>
       </c>
       <c r="I20" t="n">
-        <v>98</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.00000000113284942497894</v>
+        <v>-0.000000000920636808726804</v>
       </c>
       <c r="D21" t="n">
-        <v>0.000000000327705935938465</v>
+        <v>0.00000000007355211036705</v>
       </c>
       <c r="E21" t="n">
-        <v>-12.2330235031243</v>
+        <v>-13.2367059370623</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0805149381710006</v>
+        <v>0.0912528040541048</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.0566865396159357</v>
+        <v>-0.0616915886451893</v>
       </c>
       <c r="H21" t="n">
-        <v>0.000397582829778636</v>
+        <v>0.000453792025294844</v>
       </c>
       <c r="I21" t="n">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" t="s">
-        <v>16</v>
-      </c>
-      <c r="C22" t="n">
-        <v>-0.000000000874942639156718</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0.000000000251393004444739</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-10.9001650055631</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0.0646591992257006</v>
-      </c>
-      <c r="G22" t="n">
-        <v>-0.0501341691655996</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0.000314661348782637</v>
-      </c>
-      <c r="I22" t="n">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>19</v>
-      </c>
-      <c r="B23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C23" t="n">
-        <v>-0.00000000520693650759922</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0.00000000041839707087581</v>
-      </c>
-      <c r="E23" t="n">
-        <v>-28.1665669334067</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0.381536838631078</v>
-      </c>
-      <c r="G23" t="n">
-        <v>-0.144372698646437</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.00228015145786663</v>
-      </c>
-      <c r="I23" t="n">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="s">
-        <v>19</v>
-      </c>
-      <c r="B24" t="s">
-        <v>11</v>
-      </c>
-      <c r="C24" t="n">
-        <v>-0.00000000287110789505956</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0.000000000232068845738583</v>
-      </c>
-      <c r="E24" t="n">
-        <v>-21.975638509489</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.238732918197057</v>
-      </c>
-      <c r="G24" t="n">
-        <v>-0.108001931629995</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0.00131351800505018</v>
-      </c>
-      <c r="I24" t="n">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s">
-        <v>19</v>
-      </c>
-      <c r="B25" t="s">
-        <v>12</v>
-      </c>
-      <c r="C25" t="n">
-        <v>-0.00000000182021027054008</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0.000000000146852331251988</v>
-      </c>
-      <c r="E25" t="n">
-        <v>-18.0120336902386</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0.163853621564138</v>
-      </c>
-      <c r="G25" t="n">
-        <v>-0.0863491897459432</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0.000859564182326996</v>
-      </c>
-      <c r="I25" t="n">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="s">
-        <v>19</v>
-      </c>
-      <c r="B26" t="s">
-        <v>13</v>
-      </c>
-      <c r="C26" t="n">
-        <v>-0.00000000125729130997135</v>
-      </c>
-      <c r="D26" t="n">
-        <v>0.000000000100967193306608</v>
-      </c>
-      <c r="E26" t="n">
-        <v>-15.2593635143343</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0.119616550477939</v>
-      </c>
-      <c r="G26" t="n">
-        <v>-0.071957936590277</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0.00060818545475409</v>
-      </c>
-      <c r="I26" t="n">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="s">
-        <v>19</v>
-      </c>
-      <c r="B27" t="s">
-        <v>14</v>
-      </c>
-      <c r="C27" t="n">
-        <v>-0.000000000920636808726804</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0.00000000007355211036705</v>
-      </c>
-      <c r="E27" t="n">
-        <v>-13.2367059370623</v>
-      </c>
-      <c r="F27" t="n">
-        <v>0.0912528040541048</v>
-      </c>
-      <c r="G27" t="n">
-        <v>-0.0616915886451893</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0.000453792025294844</v>
-      </c>
-      <c r="I27" t="n">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="s">
-        <v>19</v>
-      </c>
-      <c r="B28" t="s">
-        <v>15</v>
-      </c>
-      <c r="C28" t="n">
-        <v>-0.000000000703282836956543</v>
-      </c>
-      <c r="D28" t="n">
-        <v>0.0000000000559126332073573</v>
-      </c>
-      <c r="E28" t="n">
-        <v>-11.6877331135838</v>
-      </c>
-      <c r="F28" t="n">
-        <v>0.071954425048699</v>
-      </c>
-      <c r="G28" t="n">
-        <v>-0.0539955678872008</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0.0003519313198679</v>
-      </c>
-      <c r="I28" t="n">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s">
-        <v>19</v>
-      </c>
-      <c r="B29" t="s">
-        <v>16</v>
-      </c>
-      <c r="C29" t="n">
-        <v>-0.000000000554760600150802</v>
-      </c>
-      <c r="D29" t="n">
-        <v>0.0000000000438897707791129</v>
-      </c>
-      <c r="E29" t="n">
-        <v>-10.4630570845384</v>
-      </c>
-      <c r="F29" t="n">
-        <v>0.0582154526505852</v>
-      </c>
-      <c r="G29" t="n">
-        <v>-0.0480083212089503</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0.000281077639206067</v>
-      </c>
-      <c r="I29" t="n">
         <v>117</v>
       </c>
     </row>
@@ -1284,103 +1046,103 @@
         <v>9</v>
       </c>
       <c r="B2" t="n">
-        <v>-0.00000000417591048371807</v>
+        <v>-0.000000005271362547422</v>
       </c>
       <c r="C2" t="n">
-        <v>0.000000000398307320050934</v>
+        <v>0.000000000547806823275968</v>
       </c>
       <c r="D2" t="n">
-        <v>-15.1929611737021</v>
+        <v>-17.1463892336847</v>
       </c>
       <c r="E2" t="n">
-        <v>0.193564900779139</v>
+        <v>0.225187362237541</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.0726169893876392</v>
+        <v>-0.0827340816894613</v>
       </c>
       <c r="G2" t="n">
-        <v>0.00102434856808999</v>
+        <v>0.00120572797499709</v>
       </c>
       <c r="H2" t="n">
-        <v>889</v>
+        <v>635</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.00000000126569235111904</v>
+        <v>-0.00000000165532603721674</v>
       </c>
       <c r="C3" t="n">
-        <v>0.000000000177298761385545</v>
+        <v>0.000000000232386765519311</v>
       </c>
       <c r="D3" t="n">
-        <v>-21.0933107994308</v>
+        <v>-24.541535486863</v>
       </c>
       <c r="E3" t="n">
-        <v>0.931934898902072</v>
+        <v>1.04974572349161</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.10612149296962</v>
+        <v>-0.125419152145658</v>
       </c>
       <c r="G3" t="n">
-        <v>0.00551705757488237</v>
+        <v>0.00639621921866563</v>
       </c>
       <c r="H3" t="n">
-        <v>98</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.00000000347382807854553</v>
+        <v>-0.00000000446180089713661</v>
       </c>
       <c r="C4" t="n">
-        <v>0.00000000047872682415761</v>
+        <v>0.000000000660065392455743</v>
       </c>
       <c r="D4" t="n">
-        <v>-18.2744293269652</v>
+        <v>-20.9575633560138</v>
       </c>
       <c r="E4" t="n">
-        <v>0.272957392084692</v>
+        <v>0.306271366882927</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0894267555167036</v>
+        <v>-0.103833315967078</v>
       </c>
       <c r="G4" t="n">
-        <v>0.00153285479628087</v>
+        <v>0.0017616722643256</v>
       </c>
       <c r="H4" t="n">
-        <v>686</v>
+        <v>490</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.00000000190488946128634</v>
+        <v>-0.0000000024152365583794</v>
       </c>
       <c r="C5" t="n">
-        <v>0.000000000091510691063535</v>
+        <v>0.000000000121062131176298</v>
       </c>
       <c r="D5" t="n">
-        <v>-16.971585540379</v>
+        <v>-19.3300617169062</v>
       </c>
       <c r="E5" t="n">
-        <v>0.216682394674058</v>
+        <v>0.241114077835117</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.082053890621999</v>
+        <v>-0.0944746690515683</v>
       </c>
       <c r="G5" t="n">
-        <v>0.00118330245494271</v>
+        <v>0.00134422806719034</v>
       </c>
       <c r="H5" t="n">
-        <v>819</v>
+        <v>585</v>
       </c>
     </row>
   </sheetData>

</xml_diff>